<commit_message>
added ablitiy to delete an item and the ablitiy to check item inventory across previous years
</commit_message>
<xml_diff>
--- a/Sample Data/INV-REPORT.xlsx
+++ b/Sample Data/INV-REPORT.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="30">
   <si>
     <t xml:space="preserve">رقم الصنف</t>
   </si>
@@ -109,6 +109,9 @@
   </si>
   <si>
     <t xml:space="preserve">SOLENOID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLK-320</t>
   </si>
 </sst>
 </file>
@@ -198,16 +201,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -403,273 +410,281 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:H12"/>
+  <dimension ref="A2:H13"/>
   <sheetFormatPr defaultColWidth="8.6171875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="32.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="5.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="5.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="6.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="5.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="5.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="6.62"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="0" t="n">
+      <c r="C3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="1" t="n">
         <v>34</v>
       </c>
-      <c r="E3" s="0" t="n">
+      <c r="E3" s="1" t="n">
         <v>44</v>
       </c>
-      <c r="F3" s="0" t="n">
+      <c r="F3" s="1" t="n">
         <v>73</v>
       </c>
-      <c r="G3" s="0" t="n">
+      <c r="G3" s="1" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="0" t="n">
+      <c r="C4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="1" t="n">
         <v>89</v>
       </c>
-      <c r="E4" s="0" t="n">
+      <c r="E4" s="1" t="n">
         <v>2328</v>
       </c>
-      <c r="F4" s="0" t="n">
+      <c r="F4" s="1" t="n">
         <v>2152</v>
       </c>
-      <c r="G4" s="0" t="n">
+      <c r="G4" s="1" t="n">
         <v>265</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="0" t="n">
+      <c r="C5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="E5" s="0" t="n">
+      <c r="E5" s="1" t="n">
         <v>41</v>
       </c>
-      <c r="F5" s="0" t="n">
+      <c r="F5" s="1" t="n">
         <v>37</v>
       </c>
-      <c r="G5" s="0" t="n">
+      <c r="G5" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="0" t="n">
+      <c r="C6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="1" t="n">
         <v>549</v>
       </c>
-      <c r="E6" s="0" t="n">
+      <c r="E6" s="1" t="n">
         <v>1938</v>
       </c>
-      <c r="F6" s="0" t="n">
+      <c r="F6" s="1" t="n">
         <v>2161</v>
       </c>
-      <c r="G6" s="0" t="n">
+      <c r="G6" s="1" t="n">
         <v>326</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="0" t="n">
+      <c r="C7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="1" t="n">
         <v>163</v>
       </c>
-      <c r="E7" s="0" t="n">
+      <c r="E7" s="1" t="n">
         <v>341</v>
       </c>
-      <c r="F7" s="0" t="n">
+      <c r="F7" s="1" t="n">
         <v>500</v>
       </c>
-      <c r="G7" s="0" t="n">
+      <c r="G7" s="1" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="E8" s="0" t="n">
+      <c r="C8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="0" t="n">
+      <c r="F8" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="G8" s="0" t="n">
+      <c r="G8" s="1" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="0" t="n">
+      <c r="C9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="0" t="n">
+      <c r="E9" s="1" t="n">
         <v>121</v>
       </c>
-      <c r="F9" s="0" t="n">
+      <c r="F9" s="1" t="n">
         <v>56</v>
       </c>
-      <c r="G9" s="0" t="n">
+      <c r="G9" s="1" t="n">
         <v>65</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="0" t="n">
+      <c r="C10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="1" t="n">
         <v>34</v>
       </c>
-      <c r="E10" s="0" t="n">
+      <c r="E10" s="1" t="n">
         <v>26</v>
       </c>
-      <c r="F10" s="0" t="n">
+      <c r="F10" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="G10" s="0" t="n">
+      <c r="G10" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="0" t="n">
+      <c r="C11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="0" t="n">
+      <c r="E11" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="F11" s="0" t="n">
+      <c r="F11" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G11" s="0" t="n">
+      <c r="G11" s="1" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="0" t="n">
+      <c r="C12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="0" t="n">
+      <c r="E12" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="F12" s="0" t="n">
+      <c r="F12" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="0" t="n">
+      <c r="G12" s="1" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G13" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>